<commit_message>
convert prices from string to float for accurate chart values
</commit_message>
<xml_diff>
--- a/Dolar Tracker.xlsx
+++ b/Dolar Tracker.xlsx
@@ -153,7 +153,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'Sheet'!$B$2</f>
+              <f>'Sheet'!$B$2:$B$9</f>
             </numRef>
           </val>
         </ser>
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,18 +531,105 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>20/09/26 17:02</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1.530,00</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1.550,00</t>
-        </is>
+          <t>22/09/26 20:23</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1535</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1555</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>22/09/26 20:24</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1535</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1555</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>22/09/26 20:24</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1535</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1555</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>22/09/26 20:24</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1535</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1555</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>22/09/26 20:24</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1535</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1555</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>22/09/26 20:24</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1535</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1555</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>22/09/26 20:24</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1535</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1555</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>22/09/26 20:24</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1535</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1555</v>
       </c>
     </row>
   </sheetData>

</xml_diff>